<commit_message>
update: 减仓约 1/3 (515180 122800→40900, 159937 20600→6800, 511380 13700→4500)
</commit_message>
<xml_diff>
--- a/data/holdings.xlsx
+++ b/data/holdings.xlsx
@@ -993,7 +993,8 @@
   <cols>
     <col min="1" max="1" width="18.2222222222222" style="1" customWidth="1"/>
     <col min="2" max="2" width="13.5555555555556" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="9" style="1"/>
+    <col min="3" max="3" width="12.8888888888889" style="1"/>
+    <col min="4" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:2">
@@ -1023,7 +1024,7 @@
         <v>515180</v>
       </c>
       <c r="C5" s="1">
-        <v>122800</v>
+        <v>40900</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1034,7 +1035,7 @@
         <v>159937</v>
       </c>
       <c r="C6" s="1">
-        <v>20600</v>
+        <v>6800</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1045,7 +1046,7 @@
         <v>511380</v>
       </c>
       <c r="C7" s="1">
-        <v>13700</v>
+        <v>4500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: email table column 市值 → 数量 (show share count)
</commit_message>
<xml_diff>
--- a/data/holdings.xlsx
+++ b/data/holdings.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27948" windowHeight="12420"/>
+    <workbookView windowWidth="22188" windowHeight="9180"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1002,7 +1002,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="1">
-        <v>5</v>
+        <v>652</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1024,7 +1024,7 @@
         <v>515180</v>
       </c>
       <c r="C5" s="1">
-        <v>40900</v>
+        <v>40600</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1035,7 +1035,7 @@
         <v>159937</v>
       </c>
       <c r="C6" s="1">
-        <v>6800</v>
+        <v>6900</v>
       </c>
     </row>
     <row r="7" spans="1:3">

</xml_diff>

<commit_message>
feat: migrate to 4-asset portfolio (黄金 + 红利 + 可转债 + 纳指)
- data/holdings.xlsx: add 纳斯达克ETF华夏 (513300) 17,300 股;
  rebalance to equal weight (¥50k/ETF, ¥200k total pool, 25% each)
- src/record.py: target_w = 1/len(positions) 动态等权;
  ETF_DEFS 加入 513300 纳斯达克ETF华夏
- src/chart.py / src/grid.py / src/three_pp.py: 新增，
  支持 n 资产再平衡回测 + 复合网格引擎 + matplotlib 策略图渲染
- src/fetch.py / src/notify.py: 适配 4 资产邮件摘要 + 东财通用行情
- tests/test_record.py: 17/17 passed，新增 4 资产等权 case
- README.md / index.html / app.js: 更新文档与 UI 适配 4 资产
- .github/workflows/daily.yml: 不变行为 (repository_dispatch 触发)
- requirements.txt: akshare/pandas/openpyxl/requests/matplotlib
- scripts/: 4 资产深度分析 / 3pp vs 网格 / TP basis 对比工具
- docs/correlation_analysis.md: 4 ETF 相关性研究笔记

回测 (2020-11-05 → 2026-10-13): CAGR +3.28pp / MaxDD -4.32pp
升级理由: 加纳指后真正分散 (相关性 0.12-0.27 vs 红利-可转债 0.53)
</commit_message>
<xml_diff>
--- a/data/holdings.xlsx
+++ b/data/holdings.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>现金</t>
   </si>
@@ -48,6 +48,9 @@
   </si>
   <si>
     <t>可转债ETF博时</t>
+  </si>
+  <si>
+    <t>纳斯达克ETF华夏</t>
   </si>
 </sst>
 </file>
@@ -518,153 +521,153 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -988,13 +991,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A2:C7"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="6" outlineLevelCol="2"/>
+  <dimension ref="A2:C8"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="7" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="18.2222222222222" style="1" customWidth="1"/>
     <col min="2" max="2" width="13.5555555555556" style="1" customWidth="1"/>
-    <col min="3" max="3" width="12.8888888888889" style="1"/>
-    <col min="4" max="16384" width="9" style="1"/>
+    <col min="3" max="3" width="12.8888888888889" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="9" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:2">
@@ -1024,7 +1027,7 @@
         <v>515180</v>
       </c>
       <c r="C5" s="1">
-        <v>40600</v>
+        <v>34300</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1035,7 +1038,7 @@
         <v>159937</v>
       </c>
       <c r="C6" s="1">
-        <v>6900</v>
+        <v>5800</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1046,7 +1049,18 @@
         <v>511380</v>
       </c>
       <c r="C7" s="1">
-        <v>4500</v>
+        <v>3900</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1">
+        <v>513300</v>
+      </c>
+      <c r="C8" s="1">
+        <v>17300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(xlsx): user reverted 513300 (still observing high premium)
</commit_message>
<xml_diff>
--- a/data/holdings.xlsx
+++ b/data/holdings.xlsx
@@ -1,224 +1,177 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="9180"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="22188" windowHeight="9180" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
-  <si>
-    <t>现金</t>
-  </si>
-  <si>
-    <t>名称</t>
-  </si>
-  <si>
-    <t>code</t>
-  </si>
-  <si>
-    <t>数量</t>
-  </si>
-  <si>
-    <t>红利ETF易方达</t>
-  </si>
-  <si>
-    <t>黄金ETF博时</t>
-  </si>
-  <si>
-    <t>可转债ETF博时</t>
-  </si>
-  <si>
-    <t>纳斯达克ETF华夏</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="20">
     <font>
-      <sz val="11"/>
+      <name val="宋体"/>
+      <charset val="134"/>
       <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
+      <b val="1"/>
+      <color theme="3"/>
       <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
       <color theme="3"/>
+      <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
+      <b val="1"/>
       <color theme="3"/>
+      <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
+      <b val="1"/>
       <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FF3F3F76"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color rgb="FF3F3F3F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FF9C0006"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color theme="0"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="33">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -518,159 +471,159 @@
     </border>
   </borders>
   <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -726,19 +679,75 @@
     <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
-</file>
-
-<file path=xl/customStorage/customStorage.xml><?xml version="1.0" encoding="utf-8"?>
-<customStorage xmlns="https://web.wps.cn/et/2018/main">
-  <book/>
-  <sheets/>
-</customStorage>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -989,83 +998,93 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A2:C8"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="7" outlineLevelCol="2"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="7"/>
   <cols>
-    <col min="1" max="1" width="18.2222222222222" style="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5555555555556" style="1" customWidth="1"/>
-    <col min="3" max="3" width="12.8888888888889" style="1" customWidth="1"/>
-    <col min="4" max="16384" width="9" style="1" customWidth="1"/>
+    <col width="18.2222222222222" customWidth="1" style="1" min="1" max="1"/>
+    <col width="13.5555555555556" customWidth="1" style="1" min="2" max="2"/>
+    <col width="12.8888888888889" customWidth="1" style="1" min="3" max="3"/>
+    <col width="9" customWidth="1" style="1" min="4" max="16384"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:2">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1">
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>现金</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="n">
         <v>652</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
-      <c r="A4" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>3</v>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>数量</t>
+        </is>
       </c>
     </row>
-    <row r="5" spans="1:3">
-      <c r="A5" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="1">
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>红利ETF易方达</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="n">
         <v>515180</v>
       </c>
-      <c r="C5" s="1">
-        <v>34300</v>
+      <c r="C5" s="1" t="n">
+        <v>40600</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
-      <c r="A6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" s="1">
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>黄金ETF博时</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="n">
         <v>159937</v>
       </c>
-      <c r="C6" s="1">
-        <v>5800</v>
+      <c r="C6" s="1" t="n">
+        <v>6900</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" s="1">
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>可转债ETF博时</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="n">
         <v>511380</v>
       </c>
-      <c r="C7" s="1">
-        <v>3900</v>
+      <c r="C7" s="1" t="n">
+        <v>4500</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" s="1">
-        <v>513300</v>
-      </c>
-      <c r="C8" s="1">
-        <v>17300</v>
-      </c>
+    <row r="8">
+      <c r="A8" s="0" t="n"/>
+      <c r="B8" s="1" t="n"/>
+      <c r="C8" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
</xml_diff>